<commit_message>
fix: CAD-CAM weights BEIOA+BMET follow BITAC
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EYF8ZViZ52j72cGLCGYpbD
</commit_message>
<xml_diff>
--- a/data/xlsx/beioa--cad-cam-design-and-programming-mechanical.xlsx
+++ b/data/xlsx/beioa--cad-cam-design-and-programming-mechanical.xlsx
@@ -650,7 +650,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F16" s="9">
         <f>IFERROR(MIN(C16,D16)*E16/C16,0)</f>
@@ -674,7 +674,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F17" s="9">
         <f>IFERROR(MIN(C17,D17)*E17/C17,0)</f>
@@ -698,7 +698,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F18" s="9">
         <f>IFERROR(MIN(C18,D18)*E18/C18,0)</f>
@@ -746,7 +746,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F20" s="9">
         <f>IFERROR(MIN(C20,D20)*E20/C20,0)</f>
@@ -770,7 +770,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F21" s="9">
         <f>IFERROR(MIN(C21,D21)*E21/C21,0)</f>
@@ -794,7 +794,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F22" s="9">
         <f>IFERROR(MIN(C22,D22)*E22/C22,0)</f>

</xml_diff>